<commit_message>
Improve Excel chart typography spacing and numeric axes
</commit_message>
<xml_diff>
--- a/Poster_Charts.xlsx
+++ b/Poster_Charts.xlsx
@@ -12,18 +12,23 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Satisfaction correlations" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top priorities" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'Quality ratings'!$A$1:$N$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">'Satisfaction correlations'!$A$1:$N$51</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="3">'Top priorities'!$A$1:$N$51</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -35,8 +40,47 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <b val="1"/>
+      <color rgb="00173A5B"/>
+      <sz val="24"/>
+    </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <color rgb="0052697A"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <b val="1"/>
+      <color rgb="00173A5B"/>
+      <sz val="16"/>
+    </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <color rgb="00173A5B"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <color rgb="0052697A"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Nunito Sans"/>
+      <b val="1"/>
+      <color rgb="00173A5B"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -46,6 +90,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00173A5B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F0F5FB"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -69,6 +118,51 @@
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -147,24 +241,21 @@
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Mean quality rating</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="factor"/>
+          <yMode val="factor"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.31"/>
+          <y val="0.06"/>
+          <w val="0.58"/>
+          <h val="0.8"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="bar"/>
         <grouping val="clustered"/>
@@ -173,7 +264,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Quality ratings'!B1</f>
+              <f>'Quality ratings'!$B$42</f>
             </strRef>
           </tx>
           <spPr>
@@ -186,107 +277,179 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
-              <f>'Quality ratings'!$A$2:$A$7</f>
-            </numRef>
+            <strRef>
+              <f>'Quality ratings'!$A$43:$A$48</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Quality ratings'!$B$2:$B$7</f>
+              <f>'Quality ratings'!$B$43:$B$48</f>
             </numRef>
           </val>
         </ser>
         <dLbls>
           <numFmt formatCode="0.00"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1800" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="173A5B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Nunito Sans"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+              <a:endParaRPr sz="1800" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="173A5B"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
           <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
         </dLbls>
-        <gapWidth val="150"/>
+        <gapWidth val="110"/>
+        <overlap val="0"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
-          <max val="5"/>
-          <min val="0"/>
+          <orientation val="maxMin"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Mean quality rating</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1800" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="173A5B"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>None</a:t>
+            </a:r>
+            <a:endParaRPr sz="1800" b="0">
+              <a:solidFill>
+                <a:srgbClr val="173A5B"/>
+              </a:solidFill>
+              <a:latin typeface="Nunito Sans"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
-        <crosses val="max"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
-          <orientation val="maxMin"/>
+          <orientation val="minMax"/>
+          <max val="5"/>
+          <min val="0"/>
         </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <axPos val="b"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E0E7EF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1400" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="52697A"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>None</a:t>
+            </a:r>
+            <a:endParaRPr sz="1400" b="0">
+              <a:solidFill>
+                <a:srgbClr val="52697A"/>
+              </a:solidFill>
+              <a:latin typeface="Nunito Sans"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
+        <majorUnit val="1"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Pearson r with satisfaction</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="factor"/>
+          <yMode val="factor"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.31"/>
+          <y val="0.06"/>
+          <w val="0.58"/>
+          <h val="0.8"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="bar"/>
         <grouping val="clustered"/>
@@ -295,7 +458,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Satisfaction correlations'!B1</f>
+              <f>'Satisfaction correlations'!$B$42</f>
             </strRef>
           </tx>
           <spPr>
@@ -308,107 +471,179 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
-              <f>'Satisfaction correlations'!$A$2:$A$7</f>
-            </numRef>
+            <strRef>
+              <f>'Satisfaction correlations'!$A$43:$A$48</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Satisfaction correlations'!$B$2:$B$7</f>
+              <f>'Satisfaction correlations'!$B$43:$B$48</f>
             </numRef>
           </val>
         </ser>
         <dLbls>
           <numFmt formatCode="0.000"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1800" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="173A5B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Nunito Sans"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+              <a:endParaRPr sz="1800" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="173A5B"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
           <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
         </dLbls>
-        <gapWidth val="150"/>
+        <gapWidth val="110"/>
+        <overlap val="0"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
-          <max val="1"/>
-          <min val="0"/>
+          <orientation val="maxMin"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Pearson r with satisfaction</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1800" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="173A5B"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>None</a:t>
+            </a:r>
+            <a:endParaRPr sz="1800" b="0">
+              <a:solidFill>
+                <a:srgbClr val="173A5B"/>
+              </a:solidFill>
+              <a:latin typeface="Nunito Sans"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
-        <crosses val="max"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
-          <orientation val="maxMin"/>
+          <orientation val="minMax"/>
+          <max val="1"/>
+          <min val="0"/>
         </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <axPos val="b"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E0E7EF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0.0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1400" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="52697A"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>None</a:t>
+            </a:r>
+            <a:endParaRPr sz="1400" b="0">
+              <a:solidFill>
+                <a:srgbClr val="52697A"/>
+              </a:solidFill>
+              <a:latin typeface="Nunito Sans"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
+        <majorUnit val="0.2"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
 <file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
   <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>Share choosing as top priority (%)</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
     <plotArea>
+      <layout>
+        <manualLayout>
+          <layoutTarget val="inner"/>
+          <xMode val="factor"/>
+          <yMode val="factor"/>
+          <wMode val="factor"/>
+          <hMode val="factor"/>
+          <x val="0.31"/>
+          <y val="0.06"/>
+          <w val="0.58"/>
+          <h val="0.8"/>
+        </manualLayout>
+      </layout>
       <barChart>
         <barDir val="bar"/>
         <grouping val="clustered"/>
@@ -417,7 +652,7 @@
           <order val="0"/>
           <tx>
             <strRef>
-              <f>'Top priorities'!B1</f>
+              <f>'Top priorities'!$B$42</f>
             </strRef>
           </tx>
           <spPr>
@@ -430,84 +665,159 @@
             </a:ln>
           </spPr>
           <cat>
-            <numRef>
-              <f>'Top priorities'!$A$2:$A$7</f>
-            </numRef>
+            <strRef>
+              <f>'Top priorities'!$A$43:$A$48</f>
+            </strRef>
           </cat>
           <val>
             <numRef>
-              <f>'Top priorities'!$B$2:$B$7</f>
+              <f>'Top priorities'!$B$43:$B$48</f>
             </numRef>
           </val>
         </ser>
         <dLbls>
-          <numFmt formatCode="0.0"/>
+          <numFmt formatCode="0.0&quot;%&quot;"/>
+          <txPr>
+            <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+            <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:pPr>
+                <a:defRPr sz="1800" b="1">
+                  <a:solidFill>
+                    <a:srgbClr val="173A5B"/>
+                  </a:solidFill>
+                  <a:latin typeface="Nunito Sans"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:r>
+                <a:t>None</a:t>
+              </a:r>
+              <a:endParaRPr sz="1800" b="1">
+                <a:solidFill>
+                  <a:srgbClr val="173A5B"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:endParaRPr>
+            </a:p>
+          </txPr>
           <dLblPos val="outEnd"/>
+          <showLegendKey val="0"/>
           <showVal val="1"/>
+          <showCatName val="0"/>
+          <showSerName val="0"/>
         </dLbls>
-        <gapWidth val="150"/>
+        <gapWidth val="110"/>
+        <overlap val="0"/>
         <axId val="10"/>
         <axId val="100"/>
       </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
-          <orientation val="minMax"/>
-          <max val="40"/>
-          <min val="0"/>
+          <orientation val="maxMin"/>
         </scaling>
         <axPos val="l"/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t>Share choosing as top priority (%)</a:t>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1800" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="173A5B"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>None</a:t>
+            </a:r>
+            <a:endParaRPr sz="1800" b="0">
+              <a:solidFill>
+                <a:srgbClr val="173A5B"/>
+              </a:solidFill>
+              <a:latin typeface="Nunito Sans"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="100"/>
-        <crosses val="max"/>
+        <crosses val="autoZero"/>
         <lblOffset val="100"/>
       </catAx>
       <valAx>
         <axId val="100"/>
         <scaling>
-          <orientation val="maxMin"/>
+          <orientation val="minMax"/>
+          <max val="40"/>
+          <min val="0"/>
         </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <title>
-          <tx>
-            <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:pPr>
-                  <a:defRPr/>
-                </a:pPr>
-                <a:r>
-                  <a:t/>
-                </a:r>
-              </a:p>
-            </rich>
-          </tx>
-        </title>
+        <axPos val="b"/>
+        <majorGridlines>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" w="9525">
+              <a:solidFill>
+                <a:srgbClr val="E0E7EF"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+        </majorGridlines>
+        <numFmt formatCode="0&quot;%&quot;" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
+        <tickLblPos val="nextTo"/>
+        <spPr>
+          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:noFill/>
+            <a:prstDash val="solid"/>
+          </a:ln>
+        </spPr>
+        <txPr>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr sz="1400" b="0">
+                <a:solidFill>
+                  <a:srgbClr val="52697A"/>
+                </a:solidFill>
+                <a:latin typeface="Nunito Sans"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:t>None</a:t>
+            </a:r>
+            <a:endParaRPr sz="1400" b="0">
+              <a:solidFill>
+                <a:srgbClr val="52697A"/>
+              </a:solidFill>
+              <a:latin typeface="Nunito Sans"/>
+            </a:endParaRPr>
+          </a:p>
+        </txPr>
         <crossAx val="10"/>
+        <crosses val="max"/>
+        <majorUnit val="10"/>
       </valAx>
     </plotArea>
     <plotVisOnly val="1"/>
     <dispBlanksAs val="gap"/>
   </chart>
+  <spPr>
+    <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:noFill/>
+      <a:prstDash val="solid"/>
+    </a:ln>
+  </spPr>
 </chartSpace>
 </file>
 
@@ -515,12 +825,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4680000"/>
+    <ext cx="11880000" cy="6840000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -542,12 +852,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4680000"/>
+    <ext cx="11880000" cy="6840000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -569,12 +879,12 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>5</col>
+      <col>0</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="8640000" cy="4680000"/>
+    <ext cx="11880000" cy="6840000"/>
     <graphicFrame>
       <nvGraphicFramePr>
         <cNvPr id="1" name="Chart 1"/>
@@ -590,6 +900,45 @@
     <clientData/>
   </oneCellAnchor>
 </wsDr>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="PosterChartData1" displayName="PosterChartData1" ref="A42:D48" headerRowCount="1">
+  <autoFilter ref="A42:D48"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Dimension"/>
+    <tableColumn id="2" name="Mean quality rating"/>
+    <tableColumn id="3" name="Sample n"/>
+    <tableColumn id="4" name="Displayed value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PosterChartData2" displayName="PosterChartData2" ref="A42:D48" headerRowCount="1">
+  <autoFilter ref="A42:D48"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Dimension"/>
+    <tableColumn id="2" name="Pearson r with satisfaction"/>
+    <tableColumn id="3" name="Sample n"/>
+    <tableColumn id="4" name="Displayed value"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="3" name="PosterChartData3" displayName="PosterChartData3" ref="A42:D48" headerRowCount="1">
+  <autoFilter ref="A42:D48"/>
+  <tableColumns count="4">
+    <tableColumn id="1" name="Dimension"/>
+    <tableColumn id="2" name="Share choosing as top priority (%)"/>
+    <tableColumn id="3" name="Sample n"/>
+    <tableColumn id="4" name="Priority count"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -881,7 +1230,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -891,86 +1240,110 @@
   </cols>
   <sheetData>
     <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="5" t="inlineStr">
         <is>
           <t>Poster charts</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Chaymae Elkasri — Economy &amp; Finance</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Contents</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="8" t="inlineStr">
         <is>
           <t>Three editable Excel charts and their source values, matching the final poster.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="3" ht="34" customHeight="1">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Sample</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="8" t="inlineStr">
         <is>
           <t>60 consenting eligible participants from 71 submissions. Return handling: 41 complete paired responses.</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="8" t="inlineStr">
         <is>
           <t>#1A7AE5 for all data bars.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="5" ht="34" customHeight="1">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Interpretation</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B5" s="8" t="inlineStr">
         <is>
           <t>Correlations show association, not causation.</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="6" ht="34" customHeight="1">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Rounding</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Means: 2 decimals; correlations: 3 decimals; priority percentages: 1 decimal.</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="7" ht="34" customHeight="1">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Top-three priorities</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="8" t="inlineStr">
         <is>
           <t>47 / 60 = 78.3%. Category shares sum to 100.1% when rounded.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Typography</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Install included Nunito Sans fonts before opening in Excel to preserve chart typography.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Chart layout</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Native horizontal bars; fixed zero-based numeric ranges 0–5, 0–1 and 0–40%; all series #1A7AE5.</t>
         </is>
       </c>
     </row>
@@ -983,157 +1356,198 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>QUALITY RATING</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Mean score on a five-point scale</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>SOURCE DATA FOR THE POSTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>Mean quality rating</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>Sample n</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Displayed value</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Order accuracy</t>
         </is>
       </c>
-      <c r="B2" s="2" t="n">
+      <c r="B43" s="14" t="n">
         <v>4.575</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C43" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>4.58</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Product condition</t>
         </is>
       </c>
-      <c r="B3" s="2" t="n">
+      <c r="B44" s="16" t="n">
         <v>4.383333333333334</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C44" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>4.38</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="B4" s="2" t="n">
+      <c r="B45" s="14" t="n">
         <v>4.358333333333333</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C45" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D45" s="13" t="inlineStr">
         <is>
           <t>4.36</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Reliability</t>
         </is>
       </c>
-      <c r="B5" s="2" t="n">
+      <c r="B46" s="16" t="n">
         <v>4.241666666666666</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C46" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>4.24</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Delivery speed</t>
         </is>
       </c>
-      <c r="B6" s="2" t="n">
+      <c r="B47" s="14" t="n">
         <v>3.9</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C47" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D47" s="13" t="inlineStr">
         <is>
           <t>3.90</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Return handling*</t>
         </is>
       </c>
-      <c r="B7" s="2" t="n">
+      <c r="B48" s="16" t="n">
         <v>3.060975609756098</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C48" s="15" t="n">
         <v>41</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>3.06</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>* Return handling requires both items answered; n = 41. Other quality/correlation dimensions: n = 60.</t>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>* Return handling: 41 complete paired responses; other dimensions: n = 60.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A50:N50"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1141,157 +1555,198 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>LINK TO SATISFACTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Pearson correlation (r); association, not causation</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>SOURCE DATA FOR THE POSTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>Pearson r with satisfaction</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>Sample n</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Displayed value</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Return handling*</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B43" s="18" t="n">
         <v>0.5967406469895411</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C43" s="13" t="n">
         <v>41</v>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D43" s="13" t="inlineStr">
         <is>
           <t>0.597</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="B3" s="3" t="n">
+      <c r="B44" s="19" t="n">
         <v>0.5855758537329454</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C44" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D44" s="15" t="inlineStr">
         <is>
           <t>0.586</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>Product condition</t>
         </is>
       </c>
-      <c r="B4" s="3" t="n">
+      <c r="B45" s="18" t="n">
         <v>0.5128494056492431</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C45" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D45" s="13" t="inlineStr">
         <is>
           <t>0.513</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Reliability</t>
         </is>
       </c>
-      <c r="B5" s="3" t="n">
+      <c r="B46" s="19" t="n">
         <v>0.4985601726713017</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C46" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D46" s="15" t="inlineStr">
         <is>
           <t>0.499</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Delivery speed</t>
         </is>
       </c>
-      <c r="B6" s="3" t="n">
+      <c r="B47" s="18" t="n">
         <v>0.4922155492288275</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C47" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D47" s="13" t="inlineStr">
         <is>
           <t>0.492</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Order accuracy</t>
         </is>
       </c>
-      <c r="B7" s="3" t="n">
+      <c r="B48" s="19" t="n">
         <v>0.469123759159607</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C48" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D48" s="15" t="inlineStr">
         <is>
           <t>0.469</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>* Return handling requires both items answered; n = 41. Other quality/correlation dimensions: n = 60.</t>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>* Return handling: 41 complete paired responses; other dimensions: n = 60.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A50:N50"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
@@ -1299,144 +1754,185 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
+    <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:N50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="32" customWidth="1" min="1" max="1"/>
-    <col width="40" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+    <row r="1" ht="42" customHeight="1">
+      <c r="A1" s="9" t="inlineStr">
+        <is>
+          <t>WHAT SHOPPERS PRIORITISE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="28" customHeight="1">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>Share selecting each dimension as their top priority; n = 60</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="11" t="inlineStr">
+        <is>
+          <t>SOURCE DATA FOR THE POSTER</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="42" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Dimension</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B42" s="12" t="inlineStr">
         <is>
           <t>Share choosing as top priority (%)</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C42" s="12" t="inlineStr">
         <is>
           <t>Sample n</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D42" s="12" t="inlineStr">
         <is>
           <t>Priority count</t>
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="43" ht="24" customHeight="1">
+      <c r="A43" s="13" t="inlineStr">
         <is>
           <t>Delivery speed</t>
         </is>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B43" s="20" t="n">
         <v>31.66666666666666</v>
       </c>
-      <c r="C2" t="n">
+      <c r="C43" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D2" t="n">
+      <c r="D43" s="13" t="n">
         <v>19</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="44" ht="24" customHeight="1">
+      <c r="A44" s="15" t="inlineStr">
         <is>
           <t>Reliability</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B44" s="21" t="n">
         <v>26.66666666666667</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C44" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D44" s="15" t="n">
         <v>16</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
+    <row r="45" ht="24" customHeight="1">
+      <c r="A45" s="13" t="inlineStr">
         <is>
           <t>Product condition</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B45" s="20" t="n">
         <v>20</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C45" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D45" s="13" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
+    <row r="46" ht="24" customHeight="1">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Order accuracy</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B46" s="21" t="n">
         <v>10</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C46" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D46" s="15" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+    <row r="47" ht="24" customHeight="1">
+      <c r="A47" s="13" t="inlineStr">
         <is>
           <t>Communication</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B47" s="20" t="n">
         <v>10</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C47" s="13" t="n">
         <v>60</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D47" s="13" t="n">
         <v>6</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="48" ht="24" customHeight="1">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Return handling</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B48" s="21" t="n">
         <v>1.666666666666667</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C48" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D48" s="15" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>One top-priority selection per participant; denominator n = 60.</t>
+    <row r="50" ht="34" customHeight="1">
+      <c r="A50" s="17" t="inlineStr">
+        <is>
+          <t>Percentages are count / 60 × 100; rounded shares sum to 100.1%. Top three: 47 / 60 = 78.3%.</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A50:N50"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A1:N1"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" gridLines="0"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="1" fitToWidth="1"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>